<commit_message>
ch1 update (small fix)
</commit_message>
<xml_diff>
--- a/chapter-1-financial-modeling.xlsx
+++ b/chapter-1-financial-modeling.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Other\learn_excel\financial-modeling-in-excel\Exercises_and_Datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E5AEABA-20CB-4720-AC03-BC665251251C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E8DB27-AF10-4C90-B12B-A9EFD49B078C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4FDF45FB-1CFF-4C45-826A-662E4B25C150}"/>
   </bookViews>
@@ -952,39 +952,39 @@
         <v>0</v>
       </c>
       <c r="F18" s="15">
-        <f>F19*Units*12</f>
+        <f t="shared" ref="F18:N18" si="1">F19*Units*12</f>
         <v>2208000</v>
       </c>
       <c r="G18" s="15">
-        <f>G19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2318400</v>
       </c>
       <c r="H18" s="15">
-        <f>H19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2434320</v>
       </c>
       <c r="I18" s="15">
-        <f>I19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2556036</v>
       </c>
       <c r="J18" s="15">
-        <f>J19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2683837.7999999998</v>
       </c>
       <c r="K18" s="15">
-        <f>K19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2818029.69</v>
       </c>
       <c r="L18" s="15">
-        <f>L19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>2958931.1745000007</v>
       </c>
       <c r="M18" s="15">
-        <f>M19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>3106877.7332250006</v>
       </c>
       <c r="N18" s="15">
-        <f>N19*Units*12</f>
+        <f t="shared" si="1"/>
         <v>3262221.6198862512</v>
       </c>
     </row>
@@ -1007,27 +1007,27 @@
         <v>2535.75</v>
       </c>
       <c r="I19" s="6">
-        <f t="shared" ref="I19:N19" si="1">H19*(1+$B$10)</f>
+        <f t="shared" ref="I19:N19" si="2">H19*(1+$B$10)</f>
         <v>2662.5374999999999</v>
       </c>
       <c r="J19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2795.6643749999998</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2935.4475937500001</v>
       </c>
       <c r="L19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3082.2199734375004</v>
       </c>
       <c r="M19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3236.3309721093756</v>
       </c>
       <c r="N19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3398.1475207148446</v>
       </c>
     </row>
@@ -1053,47 +1053,47 @@
         <v>-410784.00000000006</v>
       </c>
       <c r="D21" s="16">
-        <f t="shared" ref="D21:N21" si="2">-D18*(1-D23)</f>
+        <f t="shared" ref="D21:N21" si="3">-D18*(1-D23)</f>
         <v>0</v>
       </c>
       <c r="E21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-552000</v>
       </c>
       <c r="G21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-115920.0000000001</v>
       </c>
       <c r="H21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-121716.0000000001</v>
       </c>
       <c r="I21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-127801.80000000012</v>
       </c>
       <c r="J21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-134191.8900000001</v>
       </c>
       <c r="K21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-140901.48450000014</v>
       </c>
       <c r="L21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-147946.55872500016</v>
       </c>
       <c r="M21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-155343.88666125017</v>
       </c>
       <c r="N21" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-163111.08099431271</v>
       </c>
     </row>
@@ -1142,43 +1142,43 @@
       <c r="B23" s="23"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30">
-        <f t="shared" ref="E23:N23" si="3">E22/Units</f>
+        <f t="shared" ref="E23:N23" si="4">E22/Units</f>
         <v>0</v>
       </c>
       <c r="F23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.75</v>
       </c>
       <c r="G23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="H23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="I23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="J23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="K23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="L23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="M23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="N23" s="30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
     </row>
@@ -1208,43 +1208,43 @@
         <v>0</v>
       </c>
       <c r="E25" s="17">
-        <f t="shared" ref="E25:N25" si="4">SUM(E21,E18)*E26</f>
+        <f t="shared" ref="E25:N25" si="5">SUM(E21,E18)*E26</f>
         <v>0</v>
       </c>
       <c r="F25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>99360</v>
       </c>
       <c r="G25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>88099.199999999997</v>
       </c>
       <c r="H25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>92504.16</v>
       </c>
       <c r="I25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>97129.367999999988</v>
       </c>
       <c r="J25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>101985.83639999999</v>
       </c>
       <c r="K25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>107085.12821999998</v>
       </c>
       <c r="L25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>112439.38463100001</v>
       </c>
       <c r="M25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>118061.35386255002</v>
       </c>
       <c r="N25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>123964.42155567755</v>
       </c>
     </row>
@@ -1308,15 +1308,15 @@
         <v>903725</v>
       </c>
       <c r="C28" s="18">
-        <f t="shared" ref="C28:N28" si="5">SUM(C25,C21,C18)</f>
+        <f t="shared" ref="C28:N28" si="6">SUM(C25,C21,C18)</f>
         <v>0</v>
       </c>
       <c r="D28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="E28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="F28" s="18">
@@ -1324,35 +1324,35 @@
         <v>1755360</v>
       </c>
       <c r="G28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2290579.1999999997</v>
       </c>
       <c r="H28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2405108.1599999997</v>
       </c>
       <c r="I28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2525363.568</v>
       </c>
       <c r="J28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2651631.7463999996</v>
       </c>
       <c r="K28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2784213.33372</v>
       </c>
       <c r="L28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2923424.0004060003</v>
       </c>
       <c r="M28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3069595.2004263005</v>
       </c>
       <c r="N28" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3223074.9604476159</v>
       </c>
     </row>
@@ -1384,39 +1384,39 @@
         <v>0</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" ref="F30:N30" si="6">SUM(F18+F21)*F31</f>
+        <f t="shared" ref="F30:N30" si="7">SUM(F18+F21)*F31</f>
         <v>82800</v>
       </c>
       <c r="G30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>110124</v>
       </c>
       <c r="H30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>115630.20000000001</v>
       </c>
       <c r="I30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>121411.70999999999</v>
       </c>
       <c r="J30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>127482.29549999999</v>
       </c>
       <c r="K30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>133856.410275</v>
       </c>
       <c r="L30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>140549.23078875002</v>
       </c>
       <c r="M30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>147576.69232818752</v>
       </c>
       <c r="N30" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>154955.52694459693</v>
       </c>
     </row>
@@ -1483,43 +1483,43 @@
         <v>0</v>
       </c>
       <c r="E33" s="19">
-        <f t="shared" ref="E33:N33" si="7">SUM(E$18+E$21)*E34</f>
+        <f t="shared" ref="E33:N33" si="8">SUM(E$18+E$21)*E34</f>
         <v>0</v>
       </c>
       <c r="F33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>49680</v>
       </c>
       <c r="G33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>66074.399999999994</v>
       </c>
       <c r="H33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>69378.12</v>
       </c>
       <c r="I33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>72847.025999999983</v>
       </c>
       <c r="J33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>76489.377299999993</v>
       </c>
       <c r="K33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>80313.846164999981</v>
       </c>
       <c r="L33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>84329.53847325001</v>
       </c>
       <c r="M33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>88546.015396912509</v>
       </c>
       <c r="N33" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>92973.316166758159</v>
       </c>
     </row>
@@ -1585,43 +1585,43 @@
         <v>0</v>
       </c>
       <c r="E36" s="19">
-        <f t="shared" ref="E36:N36" si="8">(Units-E22)*E37</f>
+        <f t="shared" ref="E36:N36" si="9">(Units-E22)*E37</f>
         <v>24000</v>
       </c>
       <c r="F36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>6120</v>
       </c>
       <c r="G36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1248.48</v>
       </c>
       <c r="H36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1273.4496000000001</v>
       </c>
       <c r="I36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1298.9185920000002</v>
       </c>
       <c r="J36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1324.8969638400004</v>
       </c>
       <c r="K36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1351.3949031168004</v>
       </c>
       <c r="L36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1378.4228011791365</v>
       </c>
       <c r="M36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1405.9912572027192</v>
       </c>
       <c r="N36" s="19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1434.1110823467736</v>
       </c>
     </row>
@@ -1635,39 +1635,39 @@
         <v>300</v>
       </c>
       <c r="F37" s="5">
-        <f t="shared" ref="F37:N37" si="9">E37*(1+CostGrowth)</f>
+        <f t="shared" ref="F37:N37" si="10">E37*(1+CostGrowth)</f>
         <v>306</v>
       </c>
       <c r="G37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>312.12</v>
       </c>
       <c r="H37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>318.36240000000004</v>
       </c>
       <c r="I37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>324.72964800000005</v>
       </c>
       <c r="J37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>331.22424096000009</v>
       </c>
       <c r="K37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>337.84872577920009</v>
       </c>
       <c r="L37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>344.60570029478413</v>
       </c>
       <c r="M37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>351.49781430067981</v>
       </c>
       <c r="N37" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>358.52777058669341</v>
       </c>
     </row>
@@ -1696,43 +1696,43 @@
         <v>0</v>
       </c>
       <c r="E39" s="19">
-        <f t="shared" ref="E39:N39" si="10">$B$39*(1+CostGrowth^E16)</f>
+        <f t="shared" ref="E39:N39" si="11">$B$39*(1+CostGrowth^E16)</f>
         <v>-216833.64</v>
       </c>
       <c r="F39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212667.03279999999</v>
       </c>
       <c r="G39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212583.700656</v>
       </c>
       <c r="H39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.03401311999</v>
       </c>
       <c r="I39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.0006802624</v>
       </c>
       <c r="J39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.00001360523</v>
       </c>
       <c r="K39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.00000027212</v>
       </c>
       <c r="L39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.00000000544</v>
       </c>
       <c r="M39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582.00000000009</v>
       </c>
       <c r="N39" s="19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-212582</v>
       </c>
     </row>
@@ -1751,39 +1751,39 @@
         <v>-255103.91666666672</v>
       </c>
       <c r="F40" s="19">
-        <f t="shared" ref="F40:N40" si="11">-F41*F42</f>
+        <f t="shared" ref="F40:N40" si="12">-F41*F42</f>
         <v>-260205.99500000005</v>
       </c>
       <c r="G40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-265410.1149000001</v>
       </c>
       <c r="H40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-270718.31719800009</v>
       </c>
       <c r="I40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-276132.68354196008</v>
       </c>
       <c r="J40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-281655.33721279929</v>
       </c>
       <c r="K40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-287288.44395705522</v>
       </c>
       <c r="L40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-293034.21283619636</v>
       </c>
       <c r="M40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-298894.89709292026</v>
       </c>
       <c r="N40" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-304872.79503477871</v>
       </c>
     </row>
@@ -1835,39 +1835,39 @@
         <v>7288683.333333334</v>
       </c>
       <c r="F42" s="5">
-        <f t="shared" ref="F42:N42" si="12">E42*(1+CostGrowth)</f>
+        <f t="shared" ref="F42:N42" si="13">E42*(1+CostGrowth)</f>
         <v>7434457.0000000009</v>
       </c>
       <c r="G42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7583146.1400000015</v>
       </c>
       <c r="H42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7734809.0628000014</v>
       </c>
       <c r="I42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7889505.2440560013</v>
       </c>
       <c r="J42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8047295.3489371212</v>
       </c>
       <c r="K42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8208241.2559158634</v>
       </c>
       <c r="L42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8372406.0810341807</v>
       </c>
       <c r="M42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8539854.2026548646</v>
       </c>
       <c r="N42" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8710651.2867079619</v>
       </c>
     </row>
@@ -1895,51 +1895,51 @@
         <v>-466404</v>
       </c>
       <c r="C44" s="22">
-        <f t="shared" ref="C44:N44" si="13">SUM(C40,C39,C36,C33,C30)</f>
+        <f t="shared" ref="C44:N44" si="14">SUM(C40,C39,C36,C33,C30)</f>
         <v>0</v>
       </c>
       <c r="D44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="E44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-447937.55666666676</v>
       </c>
       <c r="F44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-334273.02780000004</v>
       </c>
       <c r="G44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-300546.9355560001</v>
       </c>
       <c r="H44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-297018.58161112008</v>
       </c>
       <c r="I44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-293157.02963022259</v>
       </c>
       <c r="J44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-288940.76746256452</v>
       </c>
       <c r="K44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-284348.79261421051</v>
       </c>
       <c r="L44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-279359.02077302267</v>
       </c>
       <c r="M44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-273948.19811061764</v>
       </c>
       <c r="N44" s="22">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-268091.84084107692</v>
       </c>
     </row>
@@ -1966,51 +1966,51 @@
         <v>437321</v>
       </c>
       <c r="C46" s="18">
-        <f t="shared" ref="C46:N46" si="14">SUM(C44,C28)</f>
+        <f t="shared" ref="C46:N46" si="15">SUM(C44,C28)</f>
         <v>0</v>
       </c>
       <c r="D46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="E46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-447937.55666666676</v>
       </c>
       <c r="F46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1421086.9722</v>
       </c>
       <c r="G46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1990032.2644439996</v>
       </c>
       <c r="H46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2108089.5783888795</v>
       </c>
       <c r="I46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2232206.5383697776</v>
       </c>
       <c r="J46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2362690.978937435</v>
       </c>
       <c r="K46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2499864.5411057896</v>
       </c>
       <c r="L46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2644064.9796329774</v>
       </c>
       <c r="M46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2795647.0023156828</v>
       </c>
       <c r="N46" s="18">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2954983.1196065391</v>
       </c>
     </row>
@@ -2043,39 +2043,39 @@
         <v>0</v>
       </c>
       <c r="F48" s="40">
-        <f t="shared" ref="F48:N48" si="15">IF($F$6=F16,$F$8,0)</f>
+        <f t="shared" ref="F48:N48" si="16">IF($F$6=F16,$F$8,0)</f>
         <v>0</v>
       </c>
       <c r="G48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="H48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="I48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="J48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="K48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="L48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="M48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="N48" s="40">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>49249718.660108991</v>
       </c>
     </row>
@@ -2144,51 +2144,51 @@
         <v>-21182</v>
       </c>
       <c r="C51" s="18">
-        <f t="shared" ref="C51:N51" si="16">SUM(C49,C48)</f>
+        <f t="shared" ref="C51:N51" si="17">SUM(C49,C48)</f>
         <v>0</v>
       </c>
       <c r="D51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>-7288683.333333334</v>
       </c>
       <c r="E51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>-2000000</v>
       </c>
       <c r="F51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="G51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="I51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="J51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="K51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="M51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="N51" s="18">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>49249718.660108991</v>
       </c>
     </row>
@@ -2210,55 +2210,55 @@
         <v>21</v>
       </c>
       <c r="B53" s="18">
-        <f>SUM(B51,B45)</f>
-        <v>-21182</v>
+        <f>SUM(B51,B46)</f>
+        <v>416139</v>
       </c>
       <c r="C53" s="18">
-        <f t="shared" ref="C53:N53" si="17">SUM(C51,C45)</f>
+        <f t="shared" ref="C53:N53" si="18">SUM(C51,C45)</f>
         <v>0</v>
       </c>
       <c r="D53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-7288683.333333334</v>
       </c>
       <c r="E53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-2000000</v>
       </c>
       <c r="F53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="G53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="H53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="I53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="J53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="K53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="L53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="M53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="N53" s="18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>49249718.660108991</v>
       </c>
     </row>

</xml_diff>